<commit_message>
Acumular historico 2026-10-02 19:58 UTC
</commit_message>
<xml_diff>
--- a/historico/historico_despachos.xlsx
+++ b/historico/historico_despachos.xlsx
@@ -8334,17 +8334,17 @@
       </c>
       <c r="F17" s="2" t="inlineStr">
         <is>
-          <t> </t>
+          <t>2026-10-02 14:41:05</t>
         </is>
       </c>
       <c r="G17" s="2" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Entregado</t>
         </is>
       </c>
       <c r="H17" s="2" t="inlineStr">
         <is>
-          <t> </t>
+          <t>Entregado a Agencia</t>
         </is>
       </c>
       <c r="I17" s="2" t="inlineStr">
@@ -8384,7 +8384,7 @@
       </c>
       <c r="P17" s="2" t="inlineStr">
         <is>
-          <t> </t>
+          <t>19</t>
         </is>
       </c>
       <c r="Q17" s="2" t="inlineStr">
@@ -8424,7 +8424,7 @@
       </c>
       <c r="X17" s="2" t="inlineStr">
         <is>
-          <t> </t>
+          <t>1</t>
         </is>
       </c>
       <c r="Y17" s="2" t="inlineStr">
@@ -8442,12 +8442,12 @@
       </c>
       <c r="AB17" s="2" t="inlineStr">
         <is>
-          <t> </t>
+          <t>19</t>
         </is>
       </c>
       <c r="AC17" s="2" t="inlineStr">
         <is>
-          <t> </t>
+          <t>1345.0</t>
         </is>
       </c>
       <c r="AD17" s="2" t="inlineStr">
@@ -8462,7 +8462,7 @@
       </c>
       <c r="AF17" s="2" t="inlineStr">
         <is>
-          <t> </t>
+          <t>2026-10-02 14:41:05</t>
         </is>
       </c>
       <c r="AG17" s="2" t="inlineStr">
@@ -8476,11 +8476,11 @@
         </is>
       </c>
       <c r="AI17" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AJ17" s="2" t="inlineStr">
         <is>
-          <t> </t>
+          <t>0</t>
         </is>
       </c>
       <c r="AK17" s="2" t="inlineStr">
@@ -8490,7 +8490,7 @@
       </c>
       <c r="AL17" s="2" t="inlineStr">
         <is>
-          <t> </t>
+          <t>https://cdn.beetrack.com/mobile_evaluations/images/MEDIA_CAPTURED_1790969900875_c5aeecdd-c625-4a9c-b0be-e8e0977bd956_MEDIA_20261002_143819_472_4a9cac6e-5e9f-46f2-8d6c-bbdc62f7eb91.jpg; https://cdn.beetrack.com/mobile_evaluations/images/MEDIA_CAPTURED_1790969904220_5f701f38-7b42-43ce-851c-998dd2259b3f_MEDIA_20261002_143822_826_d7d4a543-645a-43b1-9699-abba260024a1.jpg; https://cdn.beetrack.com/mobile_evaluations/images/1790969989823_88587928-d64d-4c39-b4a1-353079e04a91.jpg; https://cdn.beetrack.com/mobile_evaluations/images/MEDIA_CAPTURED_1790969900875_c5aeecdd-c625-4a9c-b0be-e8e0977bd956_MEDIA_20261002_143819_472_4a9cac6e-5e9f-46f2-8d6c-bbdc62f7eb91.jpg,https://cdn.beetrack.com/mobile_evaluations/images/MEDIA_CAPTURED_1790969904220_5f701f38-7b42-43ce-851c-998dd2259b3f_MEDIA_20261002_143822_826_d7d4a543-645a-43b1-9699-abba260024a1.jpg</t>
         </is>
       </c>
       <c r="AM17" s="2" t="inlineStr">
@@ -8502,10 +8502,10 @@
         <v>28.02</v>
       </c>
       <c r="AO17" s="2" t="n">
-        <v>0</v>
+        <v>-11.988658</v>
       </c>
       <c r="AP17" s="2" t="n">
-        <v>0</v>
+        <v>-77.080611</v>
       </c>
       <c r="AQ17" s="2" t="inlineStr">
         <is>
@@ -8546,7 +8546,7 @@
       </c>
       <c r="AZ17" s="2" t="inlineStr">
         <is>
-          <t> </t>
+          <t>1</t>
         </is>
       </c>
       <c r="BA17" s="2" t="n">
@@ -8692,12 +8692,12 @@
       </c>
       <c r="CF17" s="2" t="inlineStr">
         <is>
-          <t> </t>
+          <t xml:space="preserve">conforme </t>
         </is>
       </c>
       <c r="CG17" s="2" t="inlineStr">
         <is>
-          <t> </t>
+          <t>https://cdn.beetrack.com/mobile_evaluations/images/MEDIA_CAPTURED_1790969900875_c5aeecdd-c625-4a9c-b0be-e8e0977bd956_MEDIA_20261002_143819_472_4a9cac6e-5e9f-46f2-8d6c-bbdc62f7eb91.jpg</t>
         </is>
       </c>
       <c r="CH17" s="2" t="inlineStr">
@@ -8707,7 +8707,7 @@
       </c>
       <c r="CI17" s="2" t="inlineStr">
         <is>
-          <t> </t>
+          <t>https://cdn.beetrack.com/mobile_evaluations/images/1790969989823_88587928-d64d-4c39-b4a1-353079e04a91.jpg</t>
         </is>
       </c>
       <c r="CJ17" s="2" t="inlineStr">
@@ -8772,7 +8772,7 @@
       </c>
       <c r="CV17" s="2" t="inlineStr">
         <is>
-          <t> </t>
+          <t>https://cdn.beetrack.com/mobile_evaluations/images/MEDIA_CAPTURED_1790969904220_5f701f38-7b42-43ce-851c-998dd2259b3f_MEDIA_20261002_143822_826_d7d4a543-645a-43b1-9699-abba260024a1.jpg</t>
         </is>
       </c>
       <c r="CW17" s="2" t="inlineStr">
@@ -13642,7 +13642,7 @@
       </c>
       <c r="E28" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02 16:16:42</t>
+          <t>2026-10-02 15:52:26</t>
         </is>
       </c>
       <c r="F28" s="2" t="inlineStr">
@@ -17023,7 +17023,7 @@
       </c>
       <c r="E35" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02 16:15:42</t>
+          <t>2026-10-02 15:51:26</t>
         </is>
       </c>
       <c r="F35" s="2" t="inlineStr">
@@ -28132,7 +28132,7 @@
       </c>
       <c r="E58" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02 16:31:43</t>
+          <t>2026-10-02 16:07:27</t>
         </is>
       </c>
       <c r="F58" s="2" t="inlineStr">
@@ -30064,22 +30064,22 @@
       </c>
       <c r="E62" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02 15:06:49</t>
+          <t>2026-10-02 14:42:05</t>
         </is>
       </c>
       <c r="F62" s="2" t="inlineStr">
         <is>
-          <t> </t>
+          <t>2026-10-02 14:42:58</t>
         </is>
       </c>
       <c r="G62" s="2" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Entregado</t>
         </is>
       </c>
       <c r="H62" s="2" t="inlineStr">
         <is>
-          <t> </t>
+          <t>Entregado a Agencia</t>
         </is>
       </c>
       <c r="I62" s="2" t="inlineStr">
@@ -30119,22 +30119,22 @@
       </c>
       <c r="P62" s="2" t="inlineStr">
         <is>
-          <t> </t>
+          <t>11</t>
         </is>
       </c>
       <c r="Q62" s="2" t="inlineStr">
         <is>
-          <t> </t>
+          <t>-11.988624</t>
         </is>
       </c>
       <c r="R62" s="2" t="inlineStr">
         <is>
-          <t> </t>
+          <t>-77.080489</t>
         </is>
       </c>
       <c r="S62" s="2" t="inlineStr">
         <is>
-          <t> </t>
+          <t>2026-10-02 14:41:13</t>
         </is>
       </c>
       <c r="T62" s="2" t="inlineStr">
@@ -30159,7 +30159,7 @@
       </c>
       <c r="X62" s="2" t="inlineStr">
         <is>
-          <t> </t>
+          <t>1</t>
         </is>
       </c>
       <c r="Y62" s="2" t="inlineStr">
@@ -30177,12 +30177,12 @@
       </c>
       <c r="AB62" s="2" t="inlineStr">
         <is>
-          <t> </t>
+          <t>11</t>
         </is>
       </c>
       <c r="AC62" s="2" t="inlineStr">
         <is>
-          <t> </t>
+          <t>18.0</t>
         </is>
       </c>
       <c r="AD62" s="2" t="inlineStr">
@@ -30197,7 +30197,7 @@
       </c>
       <c r="AF62" s="2" t="inlineStr">
         <is>
-          <t> </t>
+          <t>2026-10-02 14:42:58</t>
         </is>
       </c>
       <c r="AG62" s="2" t="inlineStr">
@@ -30211,11 +30211,11 @@
         </is>
       </c>
       <c r="AI62" s="2" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="AJ62" s="2" t="inlineStr">
         <is>
-          <t> </t>
+          <t>0</t>
         </is>
       </c>
       <c r="AK62" s="2" t="inlineStr">
@@ -30225,7 +30225,7 @@
       </c>
       <c r="AL62" s="2" t="inlineStr">
         <is>
-          <t> </t>
+          <t>https://cdn.beetrack.com/mobile_evaluations/images/MEDIA_CAPTURED_1790970083958_201647b7-2103-483c-a913-a232afbd204a_MEDIA_20261002_144121_462_a9f0a58e-c14d-4841-94e0-5e2971103249.jpg; https://cdn.beetrack.com/mobile_evaluations/images/MEDIA_CAPTURED_1790970087172_acc19efd-b8df-4769-ab5d-b8138bb59ad2_MEDIA_20261002_144125_847_a220e4c3-7ee7-4aff-97f1-e82aaa999597.jpg; https://cdn.beetrack.com/mobile_evaluations/images/1790970099844_d089d265-d445-4a78-b89c-52e5ee655601.jpg; https://cdn.beetrack.com/mobile_evaluations/images/MEDIA_CAPTURED_1790970083958_201647b7-2103-483c-a913-a232afbd204a_MEDIA_20261002_144121_462_a9f0a58e-c14d-4841-94e0-5e2971103249.jpg,https://cdn.beetrack.com/mobile_evaluations/images/MEDIA_CAPTURED_1790970087172_acc19efd-b8df-4769-ab5d-b8138bb59ad2_MEDIA_20261002_144125_847_a220e4c3-7ee7-4aff-97f1-e82aaa999597.jpg; https://cdn.beetrack.com/mobile_evaluations/images/MEDIA_CAPTURED_1790970083958_201647b7-2103-483c-a913-a232afbd204a_MEDIA_20261002_144121_462_a9f0a58e-c14d-4841-94e0-5e2971103249.jpg; https://cdn.beetrack.com/mobile_evaluations/images/MEDIA_CAPTURED_1790970087172_acc19efd-b8df-4769-ab5d-b8138bb59ad2_MEDIA_20261002_144125_847_a220e4c3-7ee7-4aff-97f1-e82aaa999597.jpg; https://cdn.beetrack.com/mobile_evaluations/images/1790970099844_d089d265-d445-4a78-b89c-52e5ee655601.jpg; https://cdn.beetrack.com/mobile_evaluations/images/MEDIA_CAPTURED_1790970083958_201647b7-2103-483c-a913-a232afbd204a_MEDIA_20261002_144121_462_a9f0a58e-c14d-4841-94e0-5e2971103249.jpg,https://cdn.beetrack.com/mobile_evaluations/images/MEDIA_CAPTURED_1790970087172_acc19efd-b8df-4769-ab5d-b8138bb59ad2_MEDIA_20261002_144125_847_a220e4c3-7ee7-4aff-97f1-e82aaa999597.jpg</t>
         </is>
       </c>
       <c r="AM62" s="2" t="inlineStr">
@@ -30237,10 +30237,10 @@
         <v>28.02</v>
       </c>
       <c r="AO62" s="2" t="n">
-        <v>0</v>
+        <v>-11.988592</v>
       </c>
       <c r="AP62" s="2" t="n">
-        <v>0</v>
+        <v>-77.080462</v>
       </c>
       <c r="AQ62" s="2" t="inlineStr">
         <is>
@@ -30281,7 +30281,7 @@
       </c>
       <c r="AZ62" s="2" t="inlineStr">
         <is>
-          <t> </t>
+          <t>1</t>
         </is>
       </c>
       <c r="BA62" s="2" t="n">
@@ -30427,12 +30427,12 @@
       </c>
       <c r="CF62" s="2" t="inlineStr">
         <is>
-          <t> </t>
+          <t xml:space="preserve">conforme </t>
         </is>
       </c>
       <c r="CG62" s="2" t="inlineStr">
         <is>
-          <t> </t>
+          <t>https://cdn.beetrack.com/mobile_evaluations/images/MEDIA_CAPTURED_1790970083958_201647b7-2103-483c-a913-a232afbd204a_MEDIA_20261002_144121_462_a9f0a58e-c14d-4841-94e0-5e2971103249.jpg</t>
         </is>
       </c>
       <c r="CH62" s="2" t="inlineStr">
@@ -30442,7 +30442,7 @@
       </c>
       <c r="CI62" s="2" t="inlineStr">
         <is>
-          <t> </t>
+          <t>https://cdn.beetrack.com/mobile_evaluations/images/1790970099844_d089d265-d445-4a78-b89c-52e5ee655601.jpg</t>
         </is>
       </c>
       <c r="CJ62" s="2" t="inlineStr">
@@ -30507,7 +30507,7 @@
       </c>
       <c r="CV62" s="2" t="inlineStr">
         <is>
-          <t> </t>
+          <t>https://cdn.beetrack.com/mobile_evaluations/images/MEDIA_CAPTURED_1790970087172_acc19efd-b8df-4769-ab5d-b8138bb59ad2_MEDIA_20261002_144125_847_a220e4c3-7ee7-4aff-97f1-e82aaa999597.jpg</t>
         </is>
       </c>
       <c r="CW62" s="2" t="inlineStr">
@@ -37792,7 +37792,7 @@
       </c>
       <c r="E78" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02 15:41:48</t>
+          <t>2026-10-02 15:17:32</t>
         </is>
       </c>
       <c r="F78" s="2" t="inlineStr">
@@ -42622,7 +42622,7 @@
       </c>
       <c r="E88" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02 15:42:48</t>
+          <t>2026-10-02 15:18:32</t>
         </is>
       </c>
       <c r="F88" s="2" t="inlineStr">
@@ -49384,7 +49384,7 @@
       </c>
       <c r="E102" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02 15:59:37</t>
+          <t>2026-10-02 15:35:21</t>
         </is>
       </c>
       <c r="F102" s="2" t="inlineStr">
@@ -59044,7 +59044,7 @@
       </c>
       <c r="E122" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02 15:26:40</t>
+          <t>2026-10-02 15:02:24</t>
         </is>
       </c>
       <c r="F122" s="2" t="inlineStr">
@@ -60493,7 +60493,7 @@
       </c>
       <c r="E125" s="2" t="inlineStr">
         <is>
-          <t>2026-10-02 16:00:37</t>
+          <t>2026-10-02 15:36:21</t>
         </is>
       </c>
       <c r="F125" s="2" t="inlineStr">
@@ -66832,17 +66832,17 @@
       </c>
       <c r="Q138" s="2" t="inlineStr">
         <is>
-          <t> </t>
+          <t>-12.204195</t>
         </is>
       </c>
       <c r="R138" s="2" t="inlineStr">
         <is>
-          <t> </t>
+          <t>-76.933324</t>
         </is>
       </c>
       <c r="S138" s="2" t="inlineStr">
         <is>
-          <t> </t>
+          <t>2026-10-02 14:44:00</t>
         </is>
       </c>
       <c r="T138" s="2" t="inlineStr">
@@ -74505,17 +74505,17 @@
       </c>
       <c r="F154" s="2" t="inlineStr">
         <is>
-          <t> </t>
+          <t>2026-10-02 14:41:26</t>
         </is>
       </c>
       <c r="G154" s="2" t="inlineStr">
         <is>
-          <t>Pendiente</t>
+          <t>Entregado</t>
         </is>
       </c>
       <c r="H154" s="2" t="inlineStr">
         <is>
-          <t> </t>
+          <t>Entregado Cobranza</t>
         </is>
       </c>
       <c r="I154" s="2" t="inlineStr">
@@ -74555,7 +74555,7 @@
       </c>
       <c r="P154" s="2" t="inlineStr">
         <is>
-          <t> </t>
+          <t>3082</t>
         </is>
       </c>
       <c r="Q154" s="2" t="inlineStr">
@@ -74595,7 +74595,7 @@
       </c>
       <c r="X154" s="2" t="inlineStr">
         <is>
-          <t> </t>
+          <t>1</t>
         </is>
       </c>
       <c r="Y154" s="2" t="inlineStr">
@@ -74613,12 +74613,12 @@
       </c>
       <c r="AB154" s="2" t="inlineStr">
         <is>
-          <t> </t>
+          <t>3082</t>
         </is>
       </c>
       <c r="AC154" s="2" t="inlineStr">
         <is>
-          <t> </t>
+          <t>123.0</t>
         </is>
       </c>
       <c r="AD154" s="2" t="inlineStr">
@@ -74633,7 +74633,7 @@
       </c>
       <c r="AF154" s="2" t="inlineStr">
         <is>
-          <t> </t>
+          <t>2026-10-02 14:41:26</t>
         </is>
       </c>
       <c r="AG154" s="2" t="inlineStr">
@@ -74651,7 +74651,7 @@
       </c>
       <c r="AJ154" s="2" t="inlineStr">
         <is>
-          <t> </t>
+          <t>0</t>
         </is>
       </c>
       <c r="AK154" s="2" t="inlineStr">
@@ -74661,7 +74661,7 @@
       </c>
       <c r="AL154" s="2" t="inlineStr">
         <is>
-          <t> </t>
+          <t>https://cdn.beetrack.com/mobile_evaluations/images/MEDIA_CAPTURED_1790969978140_29399714-7111-43b5-9606-cdf88f1e1ee2_MEDIA_20261002_143936_135_d8195427-c3af-4ab0-b9e2-a08ffb0ecb41.jpg; https://cdn.beetrack.com/mobile_evaluations/images/MEDIA_CAPTURED_1790970031509_b1c29c80-3fc6-4dc2-8df0-ef3393a54eaa_MEDIA_20261002_144030_057_725f555c-f969-486f-b4f2-9df5ef839c46.jpg; https://cdn.beetrack.com/mobile_evaluations/images/1790970003024_dc64cd06-3aa7-4ea1-974e-258eeadd0e80.jpg; https://cdn.beetrack.com/mobile_evaluations/images/MEDIA_CAPTURED_1790970008876_c6bddbe6-8aea-4624-9bd0-a4bceb078738_MEDIA_20261002_144006_950_6f8a9f8a-9f65-4477-9cda-c58fd43c5d43.jpg; https://cdn.beetrack.com/mobile_evaluations/images/MEDIA_CAPTURED_1790969978140_29399714-7111-43b5-9606-cdf88f1e1ee2_MEDIA_20261002_143936_135_d8195427-c3af-4ab0-b9e2-a08ffb0ecb41.jpg,https://cdn.beetrack.com/mobile_evaluations/images/MEDIA_CAPTURED_1790970008876_c6bddbe6-8aea-4624-9bd0-a4bceb078738_MEDIA_20261002_144006_950_6f8a9f8a-9f65-4477-9cda-c58fd43c5d43.jpg,https://cdn.beetrack.com/mobile_evaluations/images/MEDIA_CAPTURED_1790970031509_b1c29c80-3fc6-4dc2-8df0-ef3393a54eaa_MEDIA_20261002_144030_057_725f555c-f969-486f-b4f2-9df5ef839c46.jpg</t>
         </is>
       </c>
       <c r="AM154" s="2" t="inlineStr">
@@ -74673,10 +74673,10 @@
         <v>63.03</v>
       </c>
       <c r="AO154" s="2" t="n">
-        <v>0</v>
+        <v>-11.902669</v>
       </c>
       <c r="AP154" s="2" t="n">
-        <v>0</v>
+        <v>-77.128359</v>
       </c>
       <c r="AQ154" s="2" t="inlineStr">
         <is>
@@ -74717,7 +74717,7 @@
       </c>
       <c r="AZ154" s="2" t="inlineStr">
         <is>
-          <t> </t>
+          <t>1</t>
         </is>
       </c>
       <c r="BA154" s="2" t="n">
@@ -74848,7 +74848,7 @@
       </c>
       <c r="CC154" s="2" t="inlineStr">
         <is>
-          <t> </t>
+          <t>https://cdn.beetrack.com/mobile_evaluations/images/MEDIA_CAPTURED_1790969978140_29399714-7111-43b5-9606-cdf88f1e1ee2_MEDIA_20261002_143936_135_d8195427-c3af-4ab0-b9e2-a08ffb0ecb41.jpg</t>
         </is>
       </c>
       <c r="CD154" s="2" t="inlineStr">
@@ -74863,7 +74863,7 @@
       </c>
       <c r="CF154" s="2" t="inlineStr">
         <is>
-          <t> </t>
+          <t xml:space="preserve">entregado </t>
         </is>
       </c>
       <c r="CG154" s="2" t="inlineStr">
@@ -74883,22 +74883,22 @@
       </c>
       <c r="CJ154" s="2" t="inlineStr">
         <is>
-          <t> </t>
+          <t>https://cdn.beetrack.com/mobile_evaluations/images/1790970003024_dc64cd06-3aa7-4ea1-974e-258eeadd0e80.jpg</t>
         </is>
       </c>
       <c r="CK154" s="2" t="inlineStr">
         <is>
-          <t> </t>
+          <t>Soles PEN</t>
         </is>
       </c>
       <c r="CL154" s="2" t="inlineStr">
         <is>
-          <t> </t>
+          <t>https://cdn.beetrack.com/mobile_evaluations/images/MEDIA_CAPTURED_1790970031509_b1c29c80-3fc6-4dc2-8df0-ef3393a54eaa_MEDIA_20261002_144030_057_725f555c-f969-486f-b4f2-9df5ef839c46.jpg</t>
         </is>
       </c>
       <c r="CM154" s="2" t="inlineStr">
         <is>
-          <t> </t>
+          <t>Izipay QR</t>
         </is>
       </c>
       <c r="CN154" s="2" t="inlineStr">
@@ -74928,17 +74928,17 @@
       </c>
       <c r="CS154" s="2" t="inlineStr">
         <is>
-          <t> </t>
+          <t>Bueno</t>
         </is>
       </c>
       <c r="CT154" s="2" t="inlineStr">
         <is>
-          <t> </t>
+          <t>376.30</t>
         </is>
       </c>
       <c r="CU154" s="2" t="inlineStr">
         <is>
-          <t> </t>
+          <t>https://cdn.beetrack.com/mobile_evaluations/images/MEDIA_CAPTURED_1790970008876_c6bddbe6-8aea-4624-9bd0-a4bceb078738_MEDIA_20261002_144006_950_6f8a9f8a-9f65-4477-9cda-c58fd43c5d43.jpg</t>
         </is>
       </c>
       <c r="CV154" s="2" t="inlineStr">

</xml_diff>